<commit_message>
Enhance model usage guidelines and update token usage reference.
- Expanded the model usage reference section to include new sheets for benchmarking and task fit, emphasizing their role in model selection.
- Clarified the approach to combining benchmark scores with cost and project context for model recommendations.
- Removed the outdated `cursor_model_token_usage_rates.xlsx` file and updated the existing one to reflect current usage rates.
</commit_message>
<xml_diff>
--- a/docs/model-selection/cursor_model_token_usage_rates.xlsx
+++ b/docs/model-selection/cursor_model_token_usage_rates.xlsx
@@ -2,9 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Rates" sheetId="1" r:id="R2ca615a065fb4789"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rfaefc229002742e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R6d866cbd91954a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Rates" sheetId="1" r:id="R5e64cbaa4ba04f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R75a35a33a8614f95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Guide" sheetId="3" r:id="R47ad17780d044b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Benchmark Signals" sheetId="4" r:id="Rb6b72852e5ba4055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Fit Matrix" sheetId="5" r:id="R32f099cbdec049c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R52ca84d59fd742ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,12 +18,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="$#,##0.000"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
-    <x:numFmt numFmtId="202" formatCode="0.0%"/>
+    <x:numFmt numFmtId="202" formatCode="0.0"/>
+    <x:numFmt numFmtId="203" formatCode="#,##0"/>
+    <x:numFmt numFmtId="204" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -40,10 +45,28 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
+      <x:color rgb="FFE0E7FF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFCFFAFE"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFEF3C7"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -58,6 +81,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1E3A8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF3730A3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4338CA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF164E63"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF155E75"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF713F12"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF92400E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -81,7 +134,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="25">
+  <x:borders count="49">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -133,6 +186,162 @@
       </x:right>
       <x:bottom style="thin">
         <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFC7D2FE"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFA5F3FC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFFDE68A"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFFDE68A"/>
       </x:bottom>
     </x:border>
     <x:border>
@@ -243,7 +452,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="58">
+  <x:cellXfs count="130">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -292,46 +501,192 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -364,6 +719,60 @@
     <x:tableColumn id="17" name="Source URL"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BenchmarkGuide" displayName="BenchmarkGuide" ref="A5:G16" headerRowCount="1">
+  <x:autoFilter ref="A5:G16"/>
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="Benchmark"/>
+    <x:tableColumn id="2" name="Capability Signal"/>
+    <x:tableColumn id="3" name="Best Task Fit"/>
+    <x:tableColumn id="4" name="How to Use in Recommendation"/>
+    <x:tableColumn id="5" name="Cost / Token Implication"/>
+    <x:tableColumn id="6" name="Limitations"/>
+    <x:tableColumn id="7" name="Source URL"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium5" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="BenchmarkSignals" displayName="BenchmarkSignals" ref="A5:N25" headerRowCount="1">
+  <x:autoFilter ref="A5:N25"/>
+  <x:tableColumns count="14">
+    <x:tableColumn id="1" name="Benchmark"/>
+    <x:tableColumn id="2" name="Model / Agent"/>
+    <x:tableColumn id="3" name="Cursor/Codex Mapping"/>
+    <x:tableColumn id="4" name="Score"/>
+    <x:tableColumn id="5" name="Score Unit"/>
+    <x:tableColumn id="6" name="Reported Cost $"/>
+    <x:tableColumn id="7" name="Prompt Tokens"/>
+    <x:tableColumn id="8" name="Completion Tokens"/>
+    <x:tableColumn id="9" name="Total Tokens"/>
+    <x:tableColumn id="10" name="Cost per Score Point"/>
+    <x:tableColumn id="11" name="Best Task Fit"/>
+    <x:tableColumn id="12" name="Recommendation Guidance"/>
+    <x:tableColumn id="13" name="Caveat"/>
+    <x:tableColumn id="14" name="Source URL"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TaskFitMatrix" displayName="TaskFitMatrix" ref="A5:F15" headerRowCount="1">
+  <x:autoFilter ref="A5:F15"/>
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="Task Profile"/>
+    <x:tableColumn id="2" name="Benchmark Evidence To Check"/>
+    <x:tableColumn id="3" name="Primary Capability Signal"/>
+    <x:tableColumn id="4" name="Default Recommendation Pattern"/>
+    <x:tableColumn id="5" name="Escalate When"/>
+    <x:tableColumn id="6" name="Token / Usage Control"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium3" showRowStripes="1"/>
 </x:table>
 </file>
 
@@ -4088,7 +4497,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a9518a09db84667"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90d79120a6744aef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4098,189 +4507,201 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="70" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="33" t="str">
+      <x:c r="A1" s="104" t="str">
         <x:v>Assumptions</x:v>
       </x:c>
-      <x:c r="B1" s="34"/>
-      <x:c r="C1" s="34"/>
-      <x:c r="D1" s="35"/>
+      <x:c r="B1" s="105"/>
+      <x:c r="C1" s="105"/>
+      <x:c r="D1" s="106"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="36"/>
+      <x:c r="A2" s="107"/>
       <x:c r="B2" s="17"/>
       <x:c r="C2" s="17"/>
-      <x:c r="D2" s="37"/>
-    </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="38" t="str">
+      <x:c r="D2" s="108"/>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="109" t="str">
         <x:v>As-of date</x:v>
       </x:c>
-      <x:c r="B3" s="17" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>2026-06-27</x:v>
       </x:c>
       <x:c r="C3" s="10" t="str">
         <x:v>Rates were pulled from Cursor docs during this session.</x:v>
       </x:c>
-      <x:c r="D3" s="37"/>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="38" t="str">
+      <x:c r="D3" s="108"/>
+    </x:row>
+    <x:row r="4" ht="34" customHeight="1">
+      <x:c r="A4" s="109" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="B4" s="17" t="str">
+      <x:c r="B4" s="10" t="str">
         <x:v>USD per 1M tokens</x:v>
       </x:c>
       <x:c r="C4" s="10" t="str">
         <x:v>All rate columns use this unit.</x:v>
       </x:c>
-      <x:c r="D4" s="37"/>
-    </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="38" t="str">
+      <x:c r="D4" s="108"/>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="109" t="str">
         <x:v>Uncached input share</x:v>
       </x:c>
-      <x:c r="B5" s="32" t="n">
+      <x:c r="B5" s="113" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
         <x:v>Default coding-agent mix assumption.</x:v>
       </x:c>
-      <x:c r="D5" s="37"/>
-    </x:row>
-    <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="38" t="str">
+      <x:c r="D5" s="108"/>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="109" t="str">
         <x:v>Cache write share</x:v>
       </x:c>
-      <x:c r="B6" s="32" t="n">
+      <x:c r="B6" s="113" t="n">
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>Only relevant when the provider exposes cache-write pricing.</x:v>
       </x:c>
-      <x:c r="D6" s="37"/>
-    </x:row>
-    <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="38" t="str">
+      <x:c r="D6" s="108"/>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="109" t="str">
         <x:v>Cache read share</x:v>
       </x:c>
-      <x:c r="B7" s="32" t="n">
+      <x:c r="B7" s="113" t="n">
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>Most repeated repository context often reads from cache.</x:v>
       </x:c>
-      <x:c r="D7" s="37"/>
-    </x:row>
-    <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="38" t="str">
+      <x:c r="D7" s="108"/>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="109" t="str">
         <x:v>Output share</x:v>
       </x:c>
-      <x:c r="B8" s="32" t="n">
+      <x:c r="B8" s="113" t="n">
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>Outputs are usually fewer tokens than context reads.</x:v>
       </x:c>
-      <x:c r="D8" s="37"/>
-    </x:row>
-    <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="38" t="str">
+      <x:c r="D8" s="108"/>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="109" t="str">
         <x:v>Weight sum check</x:v>
       </x:c>
-      <x:c r="B9" s="32" t="n">
+      <x:c r="B9" s="113" t="n">
         <x:f>SUM(B5:B8)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>Should equal 100%.</x:v>
       </x:c>
-      <x:c r="D9" s="37"/>
-    </x:row>
-    <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="38" t="str">
+      <x:c r="D9" s="108"/>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="109" t="str">
         <x:v>Teams Cursor Token Rate $/1M</x:v>
       </x:c>
-      <x:c r="B10" s="8" t="n">
+      <x:c r="B10" s="59" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
         <x:v>Cursor docs: Teams non-Auto agent requests add this on top.</x:v>
       </x:c>
-      <x:c r="D10" s="37"/>
-    </x:row>
-    <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="38" t="str">
+      <x:c r="D10" s="108"/>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="109" t="str">
         <x:v>Include Teams non-Auto surcharge? 1=yes, 0=no</x:v>
       </x:c>
-      <x:c r="B11" s="17" t="n">
+      <x:c r="B11" s="10" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>Default is 0 for individual-plan comparison.</x:v>
       </x:c>
-      <x:c r="D11" s="37"/>
-    </x:row>
-    <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="38" t="str">
+      <x:c r="D11" s="108"/>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="109" t="str">
         <x:v>Sort basis</x:v>
       </x:c>
-      <x:c r="B12" s="17" t="str">
+      <x:c r="B12" s="10" t="str">
         <x:v>Estimated Blended $/1M</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
         <x:v>Rows are pre-sorted by this calculated field descending.</x:v>
       </x:c>
-      <x:c r="D12" s="37"/>
-    </x:row>
-    <x:row r="13" ht="28" customHeight="1">
-      <x:c r="A13" s="38" t="str">
+      <x:c r="D12" s="108"/>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="109" t="str">
         <x:v>Blank cache write handling</x:v>
       </x:c>
-      <x:c r="B13" s="17" t="str">
+      <x:c r="B13" s="10" t="str">
         <x:v>Treated as 0 in formulas</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
         <x:v>Models without cache-write pricing are not charged for that category in this estimate.</x:v>
       </x:c>
-      <x:c r="D13" s="37"/>
-    </x:row>
-    <x:row r="14" ht="28" customHeight="1">
-      <x:c r="A14" s="38" t="str">
+      <x:c r="D13" s="108"/>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="109" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="B14" s="17" t="str">
+      <x:c r="B14" s="10" t="str">
         <x:v>https://cursor.com/docs/models-and-pricing</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
         <x:v>Plain-text URL included for auditability.</x:v>
       </x:c>
-      <x:c r="D14" s="37"/>
-    </x:row>
-    <x:row r="15" ht="28" customHeight="1">
-      <x:c r="A15" s="38" t="str">
+      <x:c r="D14" s="108"/>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="109" t="str">
         <x:v>Important caveat</x:v>
       </x:c>
-      <x:c r="B15" s="17" t="str">
+      <x:c r="B15" s="10" t="str">
         <x:v>Actual usage varies by prompt, repo size, context reuse, Max Mode, and output length.</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str"/>
-      <x:c r="D15" s="37"/>
-    </x:row>
-    <x:row r="16" ht="28" customHeight="1">
-      <x:c r="A16" s="39" t="str">
+      <x:c r="D15" s="108"/>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="109" t="str">
         <x:v>Visible vs hidden rows</x:v>
       </x:c>
-      <x:c r="B16" s="40" t="str">
+      <x:c r="B16" s="10" t="str">
         <x:v>Hidden metadata rows are retained and flagged, not removed.</x:v>
       </x:c>
-      <x:c r="C16" s="42" t="str"/>
-      <x:c r="D16" s="41"/>
+      <x:c r="C16" s="10" t="str"/>
+      <x:c r="D16" s="108"/>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="110" t="str">
+        <x:v>Benchmark source refresh date</x:v>
+      </x:c>
+      <x:c r="B17" s="114" t="str">
+        <x:v>2026-06-28</x:v>
+      </x:c>
+      <x:c r="C17" s="114" t="str">
+        <x:v>Benchmark sources were reviewed separately from rate extraction.</x:v>
+      </x:c>
+      <x:c r="D17" s="112"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4294,28 +4715,1605 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="56" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="50" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="35" t="str">
+        <x:v>Coding Benchmark Guide for Model Selection</x:v>
+      </x:c>
+      <x:c r="B1" s="36"/>
+      <x:c r="C1" s="36"/>
+      <x:c r="D1" s="36"/>
+      <x:c r="E1" s="36"/>
+      <x:c r="F1" s="36"/>
+      <x:c r="G1" s="37"/>
+    </x:row>
+    <x:row r="2" ht="46" customHeight="1">
+      <x:c r="A2" s="38" t="str">
+        <x:v>Use this sheet to match task type to benchmark evidence. Benchmarks are proxies: combine capability signal with Model Rates, task risk, verification strength, and current project guidance.</x:v>
+      </x:c>
+      <x:c r="B2" s="29"/>
+      <x:c r="C2" s="29"/>
+      <x:c r="D2" s="29"/>
+      <x:c r="E2" s="29"/>
+      <x:c r="F2" s="29"/>
+      <x:c r="G2" s="39"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="40"/>
+      <x:c r="B3" s="17"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="17"/>
+      <x:c r="G3" s="41"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="40"/>
+      <x:c r="B4" s="17"/>
+      <x:c r="C4" s="17"/>
+      <x:c r="D4" s="17"/>
+      <x:c r="E4" s="17"/>
+      <x:c r="F4" s="17"/>
+      <x:c r="G4" s="41"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="42" t="str">
+        <x:v>Benchmark</x:v>
+      </x:c>
+      <x:c r="B5" s="34" t="str">
+        <x:v>Capability Signal</x:v>
+      </x:c>
+      <x:c r="C5" s="34" t="str">
+        <x:v>Best Task Fit</x:v>
+      </x:c>
+      <x:c r="D5" s="34" t="str">
+        <x:v>How to Use in Recommendation</x:v>
+      </x:c>
+      <x:c r="E5" s="34" t="str">
+        <x:v>Cost / Token Implication</x:v>
+      </x:c>
+      <x:c r="F5" s="34" t="str">
+        <x:v>Limitations</x:v>
+      </x:c>
+      <x:c r="G5" s="43" t="str">
+        <x:v>Source URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="92" customHeight="1">
+      <x:c r="A6" s="44" t="str">
+        <x:v>CursorBench / Composer 2</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>Agentic coding score; Composer 2 reports 61.3 on CursorBench, 61.7 on Terminal-Bench, and 73.7 on SWE-bench Multilingual in the Cursor harness.</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Cursor-native agentic edits, ordinary codebase tasks, long-horizon coding inside Cursor.</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="str">
+        <x:v>Use as support for Auto/Composer when the task is low-to-moderate risk and exact model determinism is less important than included usage.</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>A specialized Cursor model can be the cheaper practical default when its capability is sufficient.</x:v>
+      </x:c>
+      <x:c r="F6" s="10" t="str">
+        <x:v>Vendor harness and Composer 2 result are proxies; do not treat as a universal model ranking.</x:v>
+      </x:c>
+      <x:c r="G6" s="45" t="str">
+        <x:v>https://arxiv.org/abs/2603.24477</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="92" customHeight="1">
+      <x:c r="A7" s="44" t="str">
+        <x:v>Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>Percent correct plus reported cost, prompt tokens, and completion tokens on 225 multi-language Exercism tasks.</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Small-to-moderate code editing, refactors, tests, and reasoning-level tradeoffs across C++, Go, Java, JavaScript, Python, and Rust.</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="str">
+        <x:v>Compare score lift against cost/token lift. Medium reasoning often gets close to high reasoning at materially lower cost.</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str">
+        <x:v>Use low/medium for scoped work; reserve high when added reliability is worth slower, heavier output.</x:v>
+      </x:c>
+      <x:c r="F7" s="10" t="str">
+        <x:v>Aider terminal harness, not Cursor; use as reasoning-tier evidence, not exact Cursor model truth.</x:v>
+      </x:c>
+      <x:c r="G7" s="45" t="str">
+        <x:v>https://aider.chat/docs/leaderboards/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="92" customHeight="1">
+      <x:c r="A8" s="44" t="str">
+        <x:v>SWE-bench Verified / Multilingual</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>% Resolved on real GitHub issue-resolution tasks; Verified has 500 human-filtered tasks and Multilingual has 300 tasks across 9 programming languages.</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Existing-repo bug fixes, regressions, cross-file refactors, and language-specific issue repair.</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str">
+        <x:v>Use to justify a predictable specific model for nontrivial repo issue work; combine with task risk and local test availability.</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>Repo issue work can spend many tokens on search, logs, and retries, so avoid top models when the task is well localized.</x:v>
+      </x:c>
+      <x:c r="F8" s="10" t="str">
+        <x:v>Benchmarks can be affected by harness and contamination; official leaderboard entries drift frequently.</x:v>
+      </x:c>
+      <x:c r="G8" s="45" t="str">
+        <x:v>https://www.swebench.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="92" customHeight="1">
+      <x:c r="A9" s="44" t="str">
+        <x:v>SWE-bench Pro</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>Pass@1 on long-horizon enterprise software tasks; paper reports GPT-5 at 23.3% and all evaluated models below 25%.</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>Broad architecture, persistence, migrations, multi-system changes, and work likely to span hours for a human engineer.</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="str">
+        <x:v>Use to justify GPT-5.5 High/Extra High, GPT-5.4 High, or Opus high tiers only when scope/risk is genuinely broad.</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str">
+        <x:v>Split tasks before escalating; high reasoning may be justified, but broad autonomous work remains low-success and token-heavy.</x:v>
+      </x:c>
+      <x:c r="F9" s="10" t="str">
+        <x:v>Commercial/held-out splits limit reproducibility; low absolute scores mean verification matters more than model rank.</x:v>
+      </x:c>
+      <x:c r="G9" s="45" t="str">
+        <x:v>https://arxiv.org/abs/2509.16941</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="92" customHeight="1">
+      <x:c r="A10" s="44" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>Terminal task-resolution accuracy across software engineering, system administration, security, ML, and data tasks.</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>Build/test failures, CI, deployment, shell-heavy debugging, data scripts, and terminal workflows.</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="str">
+        <x:v>Use high-scoring terminal-agent evidence for gnarly CLI/root-cause tasks; use cheap models for simple command execution.</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>Terminal tasks are log-heavy. Summarize outputs, cap context, and avoid MAX unless large logs/repo state are essential.</x:v>
+      </x:c>
+      <x:c r="F10" s="10" t="str">
+        <x:v>Agent harness matters heavily; model score is not separable from tooling and scaffold quality.</x:v>
+      </x:c>
+      <x:c r="G10" s="45" t="str">
+        <x:v>https://www.tbench.ai/leaderboard/terminal-bench/2.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="92" customHeight="1">
+      <x:c r="A11" s="44" t="str">
+        <x:v>BigCodeBench</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>1,140 tasks requiring multiple function calls across 139 libraries and 7 domains; best LLMs reported up to 60% versus 97% human performance.</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>Python/library/API/tool-use programming, data/web utility code, and unfamiliar package usage.</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="str">
+        <x:v>Use to prefer a coding-capable specific model when task success depends on precise library/tool usage.</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>Cheaper models are fine when APIs are familiar and tests are tight; escalate for unfamiliar libraries or weak specs.</x:v>
+      </x:c>
+      <x:c r="F11" s="10" t="str">
+        <x:v>Not a repository-edit benchmark and is mostly code-generation/tool-use oriented.</x:v>
+      </x:c>
+      <x:c r="G11" s="45" t="str">
+        <x:v>https://arxiv.org/abs/2406.15877</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="92" customHeight="1">
+      <x:c r="A12" s="44" t="str">
+        <x:v>SWE-Lancer</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>More than 1,400 real freelance software engineering tasks valued at $1M total, including independent engineering and managerial proposal-selection tasks.</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Task scoping, implementation-vs-managerial recommendations, proposal review, and economically meaningful engineering work.</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>Use to justify stronger reasoning for dev-project-manager prompts when the task includes ambiguous planning or proposal choice.</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>Managerial decomposition can save downstream tokens by avoiding the wrong implementation path.</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="str">
+        <x:v>Frontier models still fail the majority of tasks; use as a risk signal, not a guarantee.</x:v>
+      </x:c>
+      <x:c r="G12" s="45" t="str">
+        <x:v>https://openai.com/index/swe-lancer/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="92" customHeight="1">
+      <x:c r="A13" s="44" t="str">
+        <x:v>SWE-Bench Mobile</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>Production iOS benchmark with PRDs, Figma inputs, mixed Swift/Objective-C code, and comprehensive tests; best configurations report only 12% success.</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>Apple-platform UI/mobile work, especially iOS/macOS/iPadOS implementation and visual/design-driven tasks.</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>Do not rely on generic coding scores alone. Pair model choice with Xcode/iOS/macOS skills, visual checks, and narrow task boundaries.</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>A stronger model alone is not enough; workflow, simulator/Xcode verification, and task decomposition reduce wasted tokens.</x:v>
+      </x:c>
+      <x:c r="F13" s="10" t="str">
+        <x:v>Mobile-specific hosted benchmark; not a direct Cursor-model leaderboard.</x:v>
+      </x:c>
+      <x:c r="G13" s="45" t="str">
+        <x:v>https://arxiv.org/abs/2602.09540</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="92" customHeight="1">
+      <x:c r="A14" s="44" t="str">
+        <x:v>SpecBench</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>Specification-level software-engineering critique; paper reports the best performing agent, GPT-5.4, at 44.4% accuracy.</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>Architecture review, requirement ambiguity, RFC-style design critique, and pre-implementation planning.</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="str">
+        <x:v>Use stronger reasoning when the task is about finding missing/incorrect requirements before code is changed.</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>Spending more reasoning up front can save failed implementation loops for ambiguous tasks.</x:v>
+      </x:c>
+      <x:c r="F14" s="10" t="str">
+        <x:v>Evaluates specification critique rather than patch writing.</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="str">
+        <x:v>https://arxiv.org/abs/2605.30314</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="92" customHeight="1">
+      <x:c r="A15" s="44" t="str">
+        <x:v>SWE-Skills-Bench</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>Skill-injection utility and token overhead; paper reports average gain of +1.2%, 39 of 49 skills with zero pass-rate improvement, and overhead up to 451%.</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Plugin/skill recommendation discipline for coding agents.</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>Recommend only exact, domain-fit plugins/skills. Do not add skills just because they exist.</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>Unneeded skills can increase tokens without improving results; smallest useful toolset should be the default.</x:v>
+      </x:c>
+      <x:c r="F15" s="10" t="str">
+        <x:v>Skill effects depend on version fit and task/domain match.</x:v>
+      </x:c>
+      <x:c r="G15" s="45" t="str">
+        <x:v>https://arxiv.org/abs/2603.15401</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="92" customHeight="1">
+      <x:c r="A16" s="46" t="str">
+        <x:v>CORE-Bench</x:v>
+      </x:c>
+      <x:c r="B16" s="47" t="str">
+        <x:v>Repository code retrieval/localization benchmark with issue-to-edit and broader-context retrieval tasks.</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="str">
+        <x:v>Large-repo navigation, finding relevant files, and deciding whether MAX/large context is justified.</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="str">
+        <x:v>Use search/localization first; turn on MAX only when relevant context cannot be narrowed safely.</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="str">
+        <x:v>Good context selection is often cheaper than larger context windows.</x:v>
+      </x:c>
+      <x:c r="F16" s="47" t="str">
+        <x:v>Measures retrieval/localization rather than full implementation.</x:v>
+      </x:c>
+      <x:c r="G16" s="48" t="str">
+        <x:v>https://arxiv.org/abs/2606.11864</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6fe45900c614f49"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="44" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="62" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="44" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="50" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="61" t="str">
+        <x:v>Benchmark Signals</x:v>
+      </x:c>
+      <x:c r="B1" s="62"/>
+      <x:c r="C1" s="62"/>
+      <x:c r="D1" s="62"/>
+      <x:c r="E1" s="62"/>
+      <x:c r="F1" s="62"/>
+      <x:c r="G1" s="62"/>
+      <x:c r="H1" s="62"/>
+      <x:c r="I1" s="62"/>
+      <x:c r="J1" s="62"/>
+      <x:c r="K1" s="62"/>
+      <x:c r="L1" s="62"/>
+      <x:c r="M1" s="62"/>
+      <x:c r="N1" s="63"/>
+    </x:row>
+    <x:row r="2" ht="46" customHeight="1">
+      <x:c r="A2" s="64" t="str">
+        <x:v>Numeric benchmark rows and reported cost/token signals where available. Use mapping and caveats before applying any result to a Cursor or Codex model recommendation.</x:v>
+      </x:c>
+      <x:c r="B2" s="50"/>
+      <x:c r="C2" s="50"/>
+      <x:c r="D2" s="50"/>
+      <x:c r="E2" s="50"/>
+      <x:c r="F2" s="50"/>
+      <x:c r="G2" s="50"/>
+      <x:c r="H2" s="50"/>
+      <x:c r="I2" s="50"/>
+      <x:c r="J2" s="50"/>
+      <x:c r="K2" s="50"/>
+      <x:c r="L2" s="50"/>
+      <x:c r="M2" s="50"/>
+      <x:c r="N2" s="65"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="66"/>
+      <x:c r="B3" s="17"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="17"/>
+      <x:c r="G3" s="17"/>
+      <x:c r="H3" s="17"/>
+      <x:c r="I3" s="17"/>
+      <x:c r="J3" s="17"/>
+      <x:c r="K3" s="17"/>
+      <x:c r="L3" s="17"/>
+      <x:c r="M3" s="17"/>
+      <x:c r="N3" s="67"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="66"/>
+      <x:c r="B4" s="17"/>
+      <x:c r="C4" s="17"/>
+      <x:c r="D4" s="17"/>
+      <x:c r="E4" s="17"/>
+      <x:c r="F4" s="17"/>
+      <x:c r="G4" s="17"/>
+      <x:c r="H4" s="17"/>
+      <x:c r="I4" s="17"/>
+      <x:c r="J4" s="17"/>
+      <x:c r="K4" s="17"/>
+      <x:c r="L4" s="17"/>
+      <x:c r="M4" s="17"/>
+      <x:c r="N4" s="67"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="68" t="str">
+        <x:v>Benchmark</x:v>
+      </x:c>
+      <x:c r="B5" s="55" t="str">
+        <x:v>Model / Agent</x:v>
+      </x:c>
+      <x:c r="C5" s="55" t="str">
+        <x:v>Cursor/Codex Mapping</x:v>
+      </x:c>
+      <x:c r="D5" s="55" t="str">
+        <x:v>Score</x:v>
+      </x:c>
+      <x:c r="E5" s="55" t="str">
+        <x:v>Score Unit</x:v>
+      </x:c>
+      <x:c r="F5" s="55" t="str">
+        <x:v>Reported Cost $</x:v>
+      </x:c>
+      <x:c r="G5" s="55" t="str">
+        <x:v>Prompt Tokens</x:v>
+      </x:c>
+      <x:c r="H5" s="55" t="str">
+        <x:v>Completion Tokens</x:v>
+      </x:c>
+      <x:c r="I5" s="55" t="str">
+        <x:v>Total Tokens</x:v>
+      </x:c>
+      <x:c r="J5" s="55" t="str">
+        <x:v>Cost per Score Point</x:v>
+      </x:c>
+      <x:c r="K5" s="55" t="str">
+        <x:v>Best Task Fit</x:v>
+      </x:c>
+      <x:c r="L5" s="55" t="str">
+        <x:v>Recommendation Guidance</x:v>
+      </x:c>
+      <x:c r="M5" s="55" t="str">
+        <x:v>Caveat</x:v>
+      </x:c>
+      <x:c r="N5" s="69" t="str">
+        <x:v>Source URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="76" customHeight="1">
+      <x:c r="A6" s="70" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>NexAU-AHE + GPT-5.5</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>GPT-5.5 High / Extra High proxy</x:v>
+      </x:c>
+      <x:c r="D6" s="58" t="n">
+        <x:v>84.7</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>accuracy %</x:v>
+      </x:c>
+      <x:c r="F6" s="59"/>
+      <x:c r="G6" s="60"/>
+      <x:c r="H6" s="60"/>
+      <x:c r="I6" s="60" t="str">
+        <x:f>IF(COUNTA(G6:H6)=0,"",SUM(G6:H6))</x:f>
+      </x:c>
+      <x:c r="J6" s="59" t="str">
+        <x:f>IF(OR(F6="",F6=0),"",IFERROR(F6/D6,""))</x:f>
+      </x:c>
+      <x:c r="K6" s="10" t="str">
+        <x:v>Terminal-heavy coding, CI, deployment, system debugging</x:v>
+      </x:c>
+      <x:c r="L6" s="10" t="str">
+        <x:v>Top listed GPT-5.5 terminal-agent result; reserve similar tiers for difficult terminal/root-cause work.</x:v>
+      </x:c>
+      <x:c r="M6" s="10" t="str">
+        <x:v>Agent harness contributes materially.</x:v>
+      </x:c>
+      <x:c r="N6" s="71" t="str">
+        <x:v>https://www.tbench.ai/leaderboard/terminal-bench/2.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="76" customHeight="1">
+      <x:c r="A7" s="70" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>Codex CLI + GPT-5.5</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>GPT-5.5 High / Codex high proxy</x:v>
+      </x:c>
+      <x:c r="D7" s="58" t="n">
+        <x:v>82.2</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str">
+        <x:v>accuracy %</x:v>
+      </x:c>
+      <x:c r="F7" s="59"/>
+      <x:c r="G7" s="60"/>
+      <x:c r="H7" s="60"/>
+      <x:c r="I7" s="60" t="str">
+        <x:f>IF(COUNTA(G7:H7)=0,"",SUM(G7:H7))</x:f>
+      </x:c>
+      <x:c r="J7" s="59" t="str">
+        <x:f>IF(OR(F7="",F7=0),"",IFERROR(F7/D7,""))</x:f>
+      </x:c>
+      <x:c r="K7" s="10" t="str">
+        <x:v>Codex-style CLI workflows</x:v>
+      </x:c>
+      <x:c r="L7" s="10" t="str">
+        <x:v>Strong evidence for difficult CLI/debug/deployment tasks when exactness matters.</x:v>
+      </x:c>
+      <x:c r="M7" s="10" t="str">
+        <x:v>Not the same as Cursor dropdown behavior.</x:v>
+      </x:c>
+      <x:c r="N7" s="71" t="str">
+        <x:v>https://www.tbench.ai/leaderboard/terminal-bench/2.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="76" customHeight="1">
+      <x:c r="A8" s="70" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>WOZCODE + Claude Opus 4.7</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Opus 4.7 Extra High proxy</x:v>
+      </x:c>
+      <x:c r="D8" s="58" t="n">
+        <x:v>80.2</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>accuracy %</x:v>
+      </x:c>
+      <x:c r="F8" s="59"/>
+      <x:c r="G8" s="60"/>
+      <x:c r="H8" s="60"/>
+      <x:c r="I8" s="60" t="str">
+        <x:f>IF(COUNTA(G8:H8)=0,"",SUM(G8:H8))</x:f>
+      </x:c>
+      <x:c r="J8" s="59" t="str">
+        <x:f>IF(OR(F8="",F8=0),"",IFERROR(F8/D8,""))</x:f>
+      </x:c>
+      <x:c r="K8" s="10" t="str">
+        <x:v>Hard terminal workflows and broad debugging</x:v>
+      </x:c>
+      <x:c r="L8" s="10" t="str">
+        <x:v>Use only when top non-OpenAI reasoning is justified by risk or repeated failures.</x:v>
+      </x:c>
+      <x:c r="M8" s="10" t="str">
+        <x:v>Agent scaffold matters.</x:v>
+      </x:c>
+      <x:c r="N8" s="71" t="str">
+        <x:v>https://www.tbench.ai/leaderboard/terminal-bench/2.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="76" customHeight="1">
+      <x:c r="A9" s="70" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>TongAgents + Gemini 3.1 Pro</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>Gemini 3.1 Pro proxy</x:v>
+      </x:c>
+      <x:c r="D9" s="58" t="n">
+        <x:v>80.2</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str">
+        <x:v>accuracy %</x:v>
+      </x:c>
+      <x:c r="F9" s="59"/>
+      <x:c r="G9" s="60"/>
+      <x:c r="H9" s="60"/>
+      <x:c r="I9" s="60" t="str">
+        <x:f>IF(COUNTA(G9:H9)=0,"",SUM(G9:H9))</x:f>
+      </x:c>
+      <x:c r="J9" s="59" t="str">
+        <x:f>IF(OR(F9="",F9=0),"",IFERROR(F9/D9,""))</x:f>
+      </x:c>
+      <x:c r="K9" s="10" t="str">
+        <x:v>Terminal and multi-step agent tasks</x:v>
+      </x:c>
+      <x:c r="L9" s="10" t="str">
+        <x:v>Useful alternate specific-model evidence for terminal-heavy work.</x:v>
+      </x:c>
+      <x:c r="M9" s="10" t="str">
+        <x:v>Result is agent-specific.</x:v>
+      </x:c>
+      <x:c r="N9" s="71" t="str">
+        <x:v>https://www.tbench.ai/leaderboard/terminal-bench/2.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="76" customHeight="1">
+      <x:c r="A10" s="70" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>SageAgent + GPT-5.3-Codex</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>Codex 5.3 Medium proxy</x:v>
+      </x:c>
+      <x:c r="D10" s="58" t="n">
+        <x:v>78.4</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>accuracy %</x:v>
+      </x:c>
+      <x:c r="F10" s="59"/>
+      <x:c r="G10" s="60"/>
+      <x:c r="H10" s="60"/>
+      <x:c r="I10" s="60" t="str">
+        <x:f>IF(COUNTA(G10:H10)=0,"",SUM(G10:H10))</x:f>
+      </x:c>
+      <x:c r="J10" s="59" t="str">
+        <x:f>IF(OR(F10="",F10=0),"",IFERROR(F10/D10,""))</x:f>
+      </x:c>
+      <x:c r="K10" s="10" t="str">
+        <x:v>Codex coding agent tasks</x:v>
+      </x:c>
+      <x:c r="L10" s="10" t="str">
+        <x:v>Supports Codex 5.3 for substantial coding-agent work before jumping to GPT-5.5.</x:v>
+      </x:c>
+      <x:c r="M10" s="10" t="str">
+        <x:v>Agent-specific leaderboard row.</x:v>
+      </x:c>
+      <x:c r="N10" s="71" t="str">
+        <x:v>https://www.tbench.ai/leaderboard/terminal-bench/2.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="76" customHeight="1">
+      <x:c r="A11" s="70" t="str">
+        <x:v>Composer 2 Technical Report</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>Composer 2 on CursorBench</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>Composer 2.5 Fast / Auto + Composer proxy</x:v>
+      </x:c>
+      <x:c r="D11" s="58" t="n">
+        <x:v>61.3</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>benchmark score</x:v>
+      </x:c>
+      <x:c r="F11" s="59"/>
+      <x:c r="G11" s="60"/>
+      <x:c r="H11" s="60"/>
+      <x:c r="I11" s="60" t="str">
+        <x:f>IF(COUNTA(G11:H11)=0,"",SUM(G11:H11))</x:f>
+      </x:c>
+      <x:c r="J11" s="59" t="str">
+        <x:f>IF(OR(F11="",F11=0),"",IFERROR(F11/D11,""))</x:f>
+      </x:c>
+      <x:c r="K11" s="10" t="str">
+        <x:v>Cursor-native agentic coding</x:v>
+      </x:c>
+      <x:c r="L11" s="10" t="str">
+        <x:v>Supports Auto/Composer pool for everyday coding when lower cost and included usage matter.</x:v>
+      </x:c>
+      <x:c r="M11" s="10" t="str">
+        <x:v>Composer 2 report, not Composer 2.5 exact score.</x:v>
+      </x:c>
+      <x:c r="N11" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2603.24477</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="76" customHeight="1">
+      <x:c r="A12" s="70" t="str">
+        <x:v>Composer 2 Technical Report</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>Composer 2 on Terminal-Bench</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Composer / Auto terminal proxy</x:v>
+      </x:c>
+      <x:c r="D12" s="58" t="n">
+        <x:v>61.7</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>benchmark score</x:v>
+      </x:c>
+      <x:c r="F12" s="59"/>
+      <x:c r="G12" s="60"/>
+      <x:c r="H12" s="60"/>
+      <x:c r="I12" s="60" t="str">
+        <x:f>IF(COUNTA(G12:H12)=0,"",SUM(G12:H12))</x:f>
+      </x:c>
+      <x:c r="J12" s="59" t="str">
+        <x:f>IF(OR(F12="",F12=0),"",IFERROR(F12/D12,""))</x:f>
+      </x:c>
+      <x:c r="K12" s="10" t="str">
+        <x:v>Cursor terminal-agent coding</x:v>
+      </x:c>
+      <x:c r="L12" s="10" t="str">
+        <x:v>Composer-family models may be good enough for moderate terminal tasks before spending API-pool usage.</x:v>
+      </x:c>
+      <x:c r="M12" s="10" t="str">
+        <x:v>Vendor harness result.</x:v>
+      </x:c>
+      <x:c r="N12" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2603.24477</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="76" customHeight="1">
+      <x:c r="A13" s="70" t="str">
+        <x:v>Composer 2 Technical Report</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>Composer 2 on SWE-bench Multilingual</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>Composer / Auto multilingual repo proxy</x:v>
+      </x:c>
+      <x:c r="D13" s="58" t="n">
+        <x:v>73.7</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>benchmark score</x:v>
+      </x:c>
+      <x:c r="F13" s="59"/>
+      <x:c r="G13" s="60"/>
+      <x:c r="H13" s="60"/>
+      <x:c r="I13" s="60" t="str">
+        <x:f>IF(COUNTA(G13:H13)=0,"",SUM(G13:H13))</x:f>
+      </x:c>
+      <x:c r="J13" s="59" t="str">
+        <x:f>IF(OR(F13="",F13=0),"",IFERROR(F13/D13,""))</x:f>
+      </x:c>
+      <x:c r="K13" s="10" t="str">
+        <x:v>Repo issue work across languages</x:v>
+      </x:c>
+      <x:c r="L13" s="10" t="str">
+        <x:v>Use as support for Cursor-native everyday issue repair when task risk is bounded.</x:v>
+      </x:c>
+      <x:c r="M13" s="10" t="str">
+        <x:v>Vendor harness result.</x:v>
+      </x:c>
+      <x:c r="N13" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2603.24477</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="76" customHeight="1">
+      <x:c r="A14" s="70" t="str">
+        <x:v>Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>gpt-5 high</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>High reasoning proxy for GPT-5.5/GPT-5.4</x:v>
+      </x:c>
+      <x:c r="D14" s="58" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>% correct</x:v>
+      </x:c>
+      <x:c r="F14" s="59" t="n">
+        <x:v>29.0829</x:v>
+      </x:c>
+      <x:c r="G14" s="60" t="n">
+        <x:v>2675561</x:v>
+      </x:c>
+      <x:c r="H14" s="60" t="n">
+        <x:v>2623429</x:v>
+      </x:c>
+      <x:c r="I14" s="60" t="n">
+        <x:f>IF(COUNTA(G14:H14)=0,"",SUM(G14:H14))</x:f>
+        <x:v>5298990</x:v>
+      </x:c>
+      <x:c r="J14" s="59" t="n">
+        <x:f>IF(OR(F14="",F14=0),"",IFERROR(F14/D14,""))</x:f>
+        <x:v>0.3304875</x:v>
+      </x:c>
+      <x:c r="K14" s="10" t="str">
+        <x:v>Complex multi-language code editing</x:v>
+      </x:c>
+      <x:c r="L14" s="10" t="str">
+        <x:v>Highest GPT-5 reasoning row, but use only when the extra reliability is worth the added completion tokens and cost.</x:v>
+      </x:c>
+      <x:c r="M14" s="10" t="str">
+        <x:v>GPT-5 result used as reasoning-tier proxy.</x:v>
+      </x:c>
+      <x:c r="N14" s="71" t="str">
+        <x:v>https://aider.chat/docs/leaderboards/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="76" customHeight="1">
+      <x:c r="A15" s="70" t="str">
+        <x:v>Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>gpt-5 medium</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Medium reasoning proxy for GPT-5.5/GPT-5.4</x:v>
+      </x:c>
+      <x:c r="D15" s="58" t="n">
+        <x:v>86.7</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>% correct</x:v>
+      </x:c>
+      <x:c r="F15" s="59" t="n">
+        <x:v>17.693</x:v>
+      </x:c>
+      <x:c r="G15" s="60" t="n">
+        <x:v>2827261</x:v>
+      </x:c>
+      <x:c r="H15" s="60" t="n">
+        <x:v>1468799</x:v>
+      </x:c>
+      <x:c r="I15" s="60" t="n">
+        <x:f>IF(COUNTA(G15:H15)=0,"",SUM(G15:H15))</x:f>
+        <x:v>4296060</x:v>
+      </x:c>
+      <x:c r="J15" s="59" t="n">
+        <x:f>IF(OR(F15="",F15=0),"",IFERROR(F15/D15,""))</x:f>
+        <x:v>0.20407151095732412</x:v>
+      </x:c>
+      <x:c r="K15" s="10" t="str">
+        <x:v>Scoped nontrivial code editing</x:v>
+      </x:c>
+      <x:c r="L15" s="10" t="str">
+        <x:v>Only 1.3 points below high in this benchmark at materially lower reported cost and completion tokens.</x:v>
+      </x:c>
+      <x:c r="M15" s="10" t="str">
+        <x:v>GPT-5 result used as reasoning-tier proxy.</x:v>
+      </x:c>
+      <x:c r="N15" s="71" t="str">
+        <x:v>https://aider.chat/docs/leaderboards/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="76" customHeight="1">
+      <x:c r="A16" s="70" t="str">
+        <x:v>Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>gpt-5 low</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>Low reasoning proxy for Spark/Mini/low tiers</x:v>
+      </x:c>
+      <x:c r="D16" s="58" t="n">
+        <x:v>81.3</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>% correct</x:v>
+      </x:c>
+      <x:c r="F16" s="59" t="n">
+        <x:v>10.3713</x:v>
+      </x:c>
+      <x:c r="G16" s="60" t="n">
+        <x:v>2534059</x:v>
+      </x:c>
+      <x:c r="H16" s="60" t="n">
+        <x:v>779568</x:v>
+      </x:c>
+      <x:c r="I16" s="60" t="n">
+        <x:f>IF(COUNTA(G16:H16)=0,"",SUM(G16:H16))</x:f>
+        <x:v>3313627</x:v>
+      </x:c>
+      <x:c r="J16" s="59" t="n">
+        <x:f>IF(OR(F16="",F16=0),"",IFERROR(F16/D16,""))</x:f>
+        <x:v>0.12756826568265683</x:v>
+      </x:c>
+      <x:c r="K16" s="10" t="str">
+        <x:v>Cheap contained edits and tests</x:v>
+      </x:c>
+      <x:c r="L16" s="10" t="str">
+        <x:v>Strong cost-control option for well-scoped work; escalate when tests fail or ambiguity rises.</x:v>
+      </x:c>
+      <x:c r="M16" s="10" t="str">
+        <x:v>GPT-5 result used as reasoning-tier proxy.</x:v>
+      </x:c>
+      <x:c r="N16" s="71" t="str">
+        <x:v>https://aider.chat/docs/leaderboards/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="76" customHeight="1">
+      <x:c r="A17" s="70" t="str">
+        <x:v>Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>claude-opus-4-20250514 (32k thinking)</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>Opus High / Extra High proxy</x:v>
+      </x:c>
+      <x:c r="D17" s="58" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E17" s="10" t="str">
+        <x:v>% correct</x:v>
+      </x:c>
+      <x:c r="F17" s="59" t="n">
+        <x:v>65.7484</x:v>
+      </x:c>
+      <x:c r="G17" s="60" t="n">
+        <x:v>2567514</x:v>
+      </x:c>
+      <x:c r="H17" s="60" t="n">
+        <x:v>363142</x:v>
+      </x:c>
+      <x:c r="I17" s="60" t="n">
+        <x:f>IF(COUNTA(G17:H17)=0,"",SUM(G17:H17))</x:f>
+        <x:v>2930656</x:v>
+      </x:c>
+      <x:c r="J17" s="59" t="n">
+        <x:f>IF(OR(F17="",F17=0),"",IFERROR(F17/D17,""))</x:f>
+        <x:v>0.9131722222222223</x:v>
+      </x:c>
+      <x:c r="K17" s="10" t="str">
+        <x:v>Difficult review/design/code tasks</x:v>
+      </x:c>
+      <x:c r="L17" s="10" t="str">
+        <x:v>High reported cost means use top Opus tiers only when current criteria clearly justify them.</x:v>
+      </x:c>
+      <x:c r="M17" s="10" t="str">
+        <x:v>Older Opus 4 proxy, not Opus 4.7/4.8 exact.</x:v>
+      </x:c>
+      <x:c r="N17" s="71" t="str">
+        <x:v>https://aider.chat/docs/leaderboards/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="76" customHeight="1">
+      <x:c r="A18" s="70" t="str">
+        <x:v>Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>claude-sonnet-4-20250514 (32k thinking)</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="str">
+        <x:v>Sonnet Medium visual/UI proxy</x:v>
+      </x:c>
+      <x:c r="D18" s="58" t="n">
+        <x:v>61.3</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>% correct</x:v>
+      </x:c>
+      <x:c r="F18" s="59" t="n">
+        <x:v>26.5755</x:v>
+      </x:c>
+      <x:c r="G18" s="60" t="n">
+        <x:v>2863068</x:v>
+      </x:c>
+      <x:c r="H18" s="60" t="n">
+        <x:v>1271074</x:v>
+      </x:c>
+      <x:c r="I18" s="60" t="n">
+        <x:f>IF(COUNTA(G18:H18)=0,"",SUM(G18:H18))</x:f>
+        <x:v>4134142</x:v>
+      </x:c>
+      <x:c r="J18" s="59" t="n">
+        <x:f>IF(OR(F18="",F18=0),"",IFERROR(F18/D18,""))</x:f>
+        <x:v>0.4335318107667211</x:v>
+      </x:c>
+      <x:c r="K18" s="10" t="str">
+        <x:v>UI/layout and implementation with visual reasoning</x:v>
+      </x:c>
+      <x:c r="L18" s="10" t="str">
+        <x:v>Use Sonnet for UI fit, not because this coding-only score is top-ranked.</x:v>
+      </x:c>
+      <x:c r="M18" s="10" t="str">
+        <x:v>Older Sonnet 4 proxy, not Sonnet 4.6 exact.</x:v>
+      </x:c>
+      <x:c r="N18" s="71" t="str">
+        <x:v>https://aider.chat/docs/leaderboards/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="76" customHeight="1">
+      <x:c r="A19" s="70" t="str">
+        <x:v>SWE-bench Pro</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>GPT-5 under unified scaffold</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="str">
+        <x:v>GPT-5.5/GPT-5.4 High proxy</x:v>
+      </x:c>
+      <x:c r="D19" s="58" t="n">
+        <x:v>23.3</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="str">
+        <x:v>Pass@1 %</x:v>
+      </x:c>
+      <x:c r="F19" s="59"/>
+      <x:c r="G19" s="60"/>
+      <x:c r="H19" s="60"/>
+      <x:c r="I19" s="60" t="str">
+        <x:f>IF(COUNTA(G19:H19)=0,"",SUM(G19:H19))</x:f>
+      </x:c>
+      <x:c r="J19" s="59" t="str">
+        <x:f>IF(OR(F19="",F19=0),"",IFERROR(F19/D19,""))</x:f>
+      </x:c>
+      <x:c r="K19" s="10" t="str">
+        <x:v>Long-horizon enterprise software tasks</x:v>
+      </x:c>
+      <x:c r="L19" s="10" t="str">
+        <x:v>Even top models are low-success; choose stronger tiers only with decomposition and verification.</x:v>
+      </x:c>
+      <x:c r="M19" s="10" t="str">
+        <x:v>Paper result; exact Cursor model availability differs.</x:v>
+      </x:c>
+      <x:c r="N19" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2509.16941</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="76" customHeight="1">
+      <x:c r="A20" s="70" t="str">
+        <x:v>BigCodeBench</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>Best evaluated LLMs</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="str">
+        <x:v>Library/API coding proxy</x:v>
+      </x:c>
+      <x:c r="D20" s="58" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>best-model score %</x:v>
+      </x:c>
+      <x:c r="F20" s="59"/>
+      <x:c r="G20" s="60"/>
+      <x:c r="H20" s="60"/>
+      <x:c r="I20" s="60" t="str">
+        <x:f>IF(COUNTA(G20:H20)=0,"",SUM(G20:H20))</x:f>
+      </x:c>
+      <x:c r="J20" s="59" t="str">
+        <x:f>IF(OR(F20="",F20=0),"",IFERROR(F20/D20,""))</x:f>
+      </x:c>
+      <x:c r="K20" s="10" t="str">
+        <x:v>Python/library/tool-use code generation</x:v>
+      </x:c>
+      <x:c r="L20" s="10" t="str">
+        <x:v>Use stronger coding models for unfamiliar APIs or complex instruction following.</x:v>
+      </x:c>
+      <x:c r="M20" s="10" t="str">
+        <x:v>Paper rounded as up to 60%.</x:v>
+      </x:c>
+      <x:c r="N20" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2406.15877</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="76" customHeight="1">
+      <x:c r="A21" s="70" t="str">
+        <x:v>BigCodeBench</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>Human performance</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>Human reference</x:v>
+      </x:c>
+      <x:c r="D21" s="58" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="str">
+        <x:v>human score %</x:v>
+      </x:c>
+      <x:c r="F21" s="59"/>
+      <x:c r="G21" s="60"/>
+      <x:c r="H21" s="60"/>
+      <x:c r="I21" s="60" t="str">
+        <x:f>IF(COUNTA(G21:H21)=0,"",SUM(G21:H21))</x:f>
+      </x:c>
+      <x:c r="J21" s="59" t="str">
+        <x:f>IF(OR(F21="",F21=0),"",IFERROR(F21/D21,""))</x:f>
+      </x:c>
+      <x:c r="K21" s="10" t="str">
+        <x:v>Calibration reference</x:v>
+      </x:c>
+      <x:c r="L21" s="10" t="str">
+        <x:v>Large gap vs LLMs means tests/docs are still essential for API-heavy code.</x:v>
+      </x:c>
+      <x:c r="M21" s="10" t="str">
+        <x:v>Reference row, not model recommendation.</x:v>
+      </x:c>
+      <x:c r="N21" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2406.15877</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="76" customHeight="1">
+      <x:c r="A22" s="70" t="str">
+        <x:v>SWE-Bench Mobile</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>Best agent-model configurations</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="str">
+        <x:v>Apple/mobile implementation risk proxy</x:v>
+      </x:c>
+      <x:c r="D22" s="58" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="str">
+        <x:v>task success %</x:v>
+      </x:c>
+      <x:c r="F22" s="59"/>
+      <x:c r="G22" s="60"/>
+      <x:c r="H22" s="60"/>
+      <x:c r="I22" s="60" t="str">
+        <x:f>IF(COUNTA(G22:H22)=0,"",SUM(G22:H22))</x:f>
+      </x:c>
+      <x:c r="J22" s="59" t="str">
+        <x:f>IF(OR(F22="",F22=0),"",IFERROR(F22/D22,""))</x:f>
+      </x:c>
+      <x:c r="K22" s="10" t="str">
+        <x:v>iOS/macOS/iPadOS implementation and UI tasks</x:v>
+      </x:c>
+      <x:c r="L22" s="10" t="str">
+        <x:v>For Apple-platform work, model choice must be paired with Xcode/simulator/visual verification.</x:v>
+      </x:c>
+      <x:c r="M22" s="10" t="str">
+        <x:v>Best configuration success, not a specific model score.</x:v>
+      </x:c>
+      <x:c r="N22" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2602.09540</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="76" customHeight="1">
+      <x:c r="A23" s="70" t="str">
+        <x:v>SpecBench</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>Best performing agent GPT-5.4</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>GPT-5.4 Medium/High proxy</x:v>
+      </x:c>
+      <x:c r="D23" s="58" t="n">
+        <x:v>44.4</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="str">
+        <x:v>accuracy %</x:v>
+      </x:c>
+      <x:c r="F23" s="59"/>
+      <x:c r="G23" s="60"/>
+      <x:c r="H23" s="60"/>
+      <x:c r="I23" s="60" t="str">
+        <x:f>IF(COUNTA(G23:H23)=0,"",SUM(G23:H23))</x:f>
+      </x:c>
+      <x:c r="J23" s="59" t="str">
+        <x:f>IF(OR(F23="",F23=0),"",IFERROR(F23/D23,""))</x:f>
+      </x:c>
+      <x:c r="K23" s="10" t="str">
+        <x:v>Specification and architecture critique</x:v>
+      </x:c>
+      <x:c r="L23" s="10" t="str">
+        <x:v>Use stronger reasoning for ambiguous requirements before implementation.</x:v>
+      </x:c>
+      <x:c r="M23" s="10" t="str">
+        <x:v>Spec critique benchmark, not patch-writing.</x:v>
+      </x:c>
+      <x:c r="N23" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2605.30314</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="76" customHeight="1">
+      <x:c r="A24" s="70" t="str">
+        <x:v>SWE-Skills-Bench</x:v>
+      </x:c>
+      <x:c r="B24" s="10" t="str">
+        <x:v>Average skill injection gain</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>Plugin/skill selection signal</x:v>
+      </x:c>
+      <x:c r="D24" s="58" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>average pass-rate lift pp</x:v>
+      </x:c>
+      <x:c r="F24" s="59"/>
+      <x:c r="G24" s="60"/>
+      <x:c r="H24" s="60"/>
+      <x:c r="I24" s="60" t="str">
+        <x:f>IF(COUNTA(G24:H24)=0,"",SUM(G24:H24))</x:f>
+      </x:c>
+      <x:c r="J24" s="59" t="str">
+        <x:f>IF(OR(F24="",F24=0),"",IFERROR(F24/D24,""))</x:f>
+      </x:c>
+      <x:c r="K24" s="10" t="str">
+        <x:v>Plugin/skill recommendation discipline</x:v>
+      </x:c>
+      <x:c r="L24" s="10" t="str">
+        <x:v>Default to no plugin/skill unless domain fit is exact and material.</x:v>
+      </x:c>
+      <x:c r="M24" s="10" t="str">
+        <x:v>Average hides a few strong positive specialized skills.</x:v>
+      </x:c>
+      <x:c r="N24" s="71" t="str">
+        <x:v>https://arxiv.org/abs/2603.15401</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="76" customHeight="1">
+      <x:c r="A25" s="72" t="str">
+        <x:v>SWE-Skills-Bench</x:v>
+      </x:c>
+      <x:c r="B25" s="73" t="str">
+        <x:v>Maximum observed token overhead</x:v>
+      </x:c>
+      <x:c r="C25" s="73" t="str">
+        <x:v>Plugin/skill token overhead signal</x:v>
+      </x:c>
+      <x:c r="D25" s="74" t="n">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="E25" s="73" t="str">
+        <x:v>token overhead %</x:v>
+      </x:c>
+      <x:c r="F25" s="75"/>
+      <x:c r="G25" s="76"/>
+      <x:c r="H25" s="76"/>
+      <x:c r="I25" s="76" t="str">
+        <x:f>IF(COUNTA(G25:H25)=0,"",SUM(G25:H25))</x:f>
+      </x:c>
+      <x:c r="J25" s="75" t="str">
+        <x:f>IF(OR(F25="",F25=0),"",IFERROR(F25/D25,""))</x:f>
+      </x:c>
+      <x:c r="K25" s="73" t="str">
+        <x:v>Plugin/skill recommendation discipline</x:v>
+      </x:c>
+      <x:c r="L25" s="73" t="str">
+        <x:v>Avoid speculative skills because they can consume many extra tokens with no pass-rate gain.</x:v>
+      </x:c>
+      <x:c r="M25" s="73" t="str">
+        <x:v>Worst-case reported overhead.</x:v>
+      </x:c>
+      <x:c r="N25" s="77" t="str">
+        <x:v>https://arxiv.org/abs/2603.15401</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A2:N2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="D6:J25">
+    <x:cfRule type="colorScale" priority="1">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFECFEFF"/>
+        <x:color rgb="FFFEF9C3"/>
+        <x:color rgb="FFFEE2E2"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd8ceacebf0a476d"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="85" t="str">
+        <x:v>Task Fit Matrix</x:v>
+      </x:c>
+      <x:c r="B1" s="86"/>
+      <x:c r="C1" s="86"/>
+      <x:c r="D1" s="86"/>
+      <x:c r="E1" s="86"/>
+      <x:c r="F1" s="87"/>
+    </x:row>
+    <x:row r="2" ht="46" customHeight="1">
+      <x:c r="A2" s="88" t="str">
+        <x:v>Start from task profile, then select the least expensive model likely to succeed. Escalate only when benchmark evidence, task risk, ambiguity, or verification weakness justify the added token/API usage.</x:v>
+      </x:c>
+      <x:c r="B2" s="79"/>
+      <x:c r="C2" s="79"/>
+      <x:c r="D2" s="79"/>
+      <x:c r="E2" s="79"/>
+      <x:c r="F2" s="89"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="90"/>
+      <x:c r="B3" s="17"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="91"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="90"/>
+      <x:c r="B4" s="17"/>
+      <x:c r="C4" s="17"/>
+      <x:c r="D4" s="17"/>
+      <x:c r="E4" s="17"/>
+      <x:c r="F4" s="91"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="92" t="str">
+        <x:v>Task Profile</x:v>
+      </x:c>
+      <x:c r="B5" s="84" t="str">
+        <x:v>Benchmark Evidence To Check</x:v>
+      </x:c>
+      <x:c r="C5" s="84" t="str">
+        <x:v>Primary Capability Signal</x:v>
+      </x:c>
+      <x:c r="D5" s="84" t="str">
+        <x:v>Default Recommendation Pattern</x:v>
+      </x:c>
+      <x:c r="E5" s="84" t="str">
+        <x:v>Escalate When</x:v>
+      </x:c>
+      <x:c r="F5" s="93" t="str">
+        <x:v>Token / Usage Control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="80" customHeight="1">
+      <x:c r="A6" s="94" t="str">
+        <x:v>Trivial single-file edit, copy change, formatting</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>Aider low reasoning + Model Rates</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Low reasoning can still solve many scoped edits.</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="str">
+        <x:v>Cursor Auto, Composer 2.5 Fast, GPT-5.3-Codex-Spark Low, or GPT-5.4 Mini Low.</x:v>
+      </x:c>
+      <x:c r="E6" s="10" t="str">
+        <x:v>Only escalate if the file is risky, tests repeatedly fail, or hidden coupling appears.</x:v>
+      </x:c>
+      <x:c r="F6" s="95" t="str">
+        <x:v>Keep MAX off; avoid broad repo reads; preserve existing changes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="80" customHeight="1">
+      <x:c r="A7" s="94" t="str">
+        <x:v>Contained coding task with tests</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>Aider Polyglot, SWE-bench Verified</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Need reliable code editing but scope is bounded.</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="str">
+        <x:v>Auto when exact model is not important; Codex 5.3 Medium or GPT-5.4 Mini Medium when predictability matters.</x:v>
+      </x:c>
+      <x:c r="E7" s="10" t="str">
+        <x:v>Escalate to GPT-5.4 Medium/High if failures reveal unclear behavior or multi-module coupling.</x:v>
+      </x:c>
+      <x:c r="F7" s="95" t="str">
+        <x:v>Use targeted search and run focused tests; summarize logs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="80" customHeight="1">
+      <x:c r="A8" s="94" t="str">
+        <x:v>Moderate multi-file implementation or refactor</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>SWE-bench Verified / Multilingual, Aider medium</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Repository issue resolution and cross-file consistency.</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str">
+        <x:v>GPT-5.4 Medium or Codex 5.3 Medium before GPT-5.5.</x:v>
+      </x:c>
+      <x:c r="E8" s="10" t="str">
+        <x:v>Escalate when root cause is unclear, changes touch shared contracts, or test surface is broad.</x:v>
+      </x:c>
+      <x:c r="F8" s="95" t="str">
+        <x:v>Keep MAX off unless relevant context cannot be localized.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="80" customHeight="1">
+      <x:c r="A9" s="94" t="str">
+        <x:v>Terminal-heavy build, CI, deployment, or system debugging</x:v>
+      </x:c>
+      <x:c r="B9" s="10" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="C9" s="10" t="str">
+        <x:v>Command execution, environment diagnosis, and long log interpretation.</x:v>
+      </x:c>
+      <x:c r="D9" s="10" t="str">
+        <x:v>Codex 5.3 Medium/High or GPT-5.5 High for high-risk production/debugging; cheaper models for simple commands.</x:v>
+      </x:c>
+      <x:c r="E9" s="10" t="str">
+        <x:v>Escalate when failures are nondeterministic, deployment-affecting, or security-sensitive.</x:v>
+      </x:c>
+      <x:c r="F9" s="95" t="str">
+        <x:v>Cap logs, quote only key lines, and avoid live/credit-consuming requests without approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="80" customHeight="1">
+      <x:c r="A10" s="94" t="str">
+        <x:v>Live API, security, auth, secrets, or production deployment</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>Terminal-Bench 2.0, SWE-Lancer, SWE-bench Pro</x:v>
+      </x:c>
+      <x:c r="C10" s="10" t="str">
+        <x:v>High consequence and multi-system coordination.</x:v>
+      </x:c>
+      <x:c r="D10" s="10" t="str">
+        <x:v>GPT-5.5 High; Extra High only for broad unresolved root-cause or migration work.</x:v>
+      </x:c>
+      <x:c r="E10" s="10" t="str">
+        <x:v>Escalation is justified by production risk, not just task size.</x:v>
+      </x:c>
+      <x:c r="F10" s="95" t="str">
+        <x:v>Never print secrets or raw env dumps; require approval for live requests.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="80" customHeight="1">
+      <x:c r="A11" s="94" t="str">
+        <x:v>Architecture, persistence, migrations, broad planning, or proposal selection</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>SWE-bench Pro, SWE-Lancer, SpecBench</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>Long-horizon reasoning and requirement critique.</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="str">
+        <x:v>GPT-5.4 High or GPT-5.5 High; Opus High/Extra High only for difficult design/review where current criteria justify it.</x:v>
+      </x:c>
+      <x:c r="E11" s="10" t="str">
+        <x:v>Escalate when requirements are ambiguous, irreversible, or cross-system.</x:v>
+      </x:c>
+      <x:c r="F11" s="95" t="str">
+        <x:v>Split the work into phases to reduce token waste and verification risk.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="80" customHeight="1">
+      <x:c r="A12" s="94" t="str">
+        <x:v>UI, SwiftUI, Apple-platform, or mobile app work</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>SWE-Bench Mobile plus visual verification; generic coding benchmarks are weak proxies.</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Agent/workflow and verification matter as much as model strength.</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>Sonnet 4.6 Medium for visual/UI judgment, GPT-5.4 Medium for implementation, Xcode for diagnostics.</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>Escalate when UI changes span architecture, state, persistence, or repeated visual failures.</x:v>
+      </x:c>
+      <x:c r="F12" s="95" t="str">
+        <x:v>Use iOS/macOS/Xcode skills and screenshots/previews instead of MAX by default.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="80" customHeight="1">
+      <x:c r="A13" s="94" t="str">
+        <x:v>Python, data scripts, API/library integration</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>BigCodeBench, Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>Precise library use and instruction following.</x:v>
+      </x:c>
+      <x:c r="D13" s="10" t="str">
+        <x:v>GPT-5.4 Mini Medium/High or GPT-5.4 Medium depending on API unfamiliarity.</x:v>
+      </x:c>
+      <x:c r="E13" s="10" t="str">
+        <x:v>Escalate if docs are ambiguous, external systems are involved, or test oracle is weak.</x:v>
+      </x:c>
+      <x:c r="F13" s="95" t="str">
+        <x:v>Prefer official docs and focused unit tests over larger context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="80" customHeight="1">
+      <x:c r="A14" s="94" t="str">
+        <x:v>Plugin or skill recommendation inside generated prompts</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>SWE-Skills-Bench</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>Skills are useful only when matched tightly to task/domain.</x:v>
+      </x:c>
+      <x:c r="D14" s="10" t="str">
+        <x:v>Recommend None by default; add exact skills/plugins only when they materially improve verification or domain fit.</x:v>
+      </x:c>
+      <x:c r="E14" s="10" t="str">
+        <x:v>Escalate skill/plugin use when a known project or workflow-specific skill reduces risk.</x:v>
+      </x:c>
+      <x:c r="F14" s="95" t="str">
+        <x:v>Avoid speculative plugins/skills because they add token overhead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="80" customHeight="1">
+      <x:c r="A15" s="96" t="str">
+        <x:v>Large-repo localization or uncertain relevant files</x:v>
+      </x:c>
+      <x:c r="B15" s="97" t="str">
+        <x:v>CORE-Bench, SWE-bench family</x:v>
+      </x:c>
+      <x:c r="C15" s="97" t="str">
+        <x:v>Context retrieval and issue-to-edit localization.</x:v>
+      </x:c>
+      <x:c r="D15" s="97" t="str">
+        <x:v>Use repo search and targeted reads first; consider MAX only after localization fails or task requires repository-wide reasoning.</x:v>
+      </x:c>
+      <x:c r="E15" s="97" t="str">
+        <x:v>Escalate when many modules could be relevant and missing context would cause wrong edits.</x:v>
+      </x:c>
+      <x:c r="F15" s="98" t="str">
+        <x:v>Narrow context beats larger context when it preserves correctness.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfcce2f9f1fc4430"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="54" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="56" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="66" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="48" t="str">
+      <x:c r="A1" s="120" t="str">
         <x:v>Sources and Build Notes</x:v>
       </x:c>
-      <x:c r="B1" s="49"/>
-      <x:c r="C1" s="49"/>
-      <x:c r="D1" s="50"/>
+      <x:c r="B1" s="121"/>
+      <x:c r="C1" s="121"/>
+      <x:c r="D1" s="122"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="51"/>
+      <x:c r="A2" s="123"/>
       <x:c r="B2" s="17"/>
       <x:c r="C2" s="17"/>
-      <x:c r="D2" s="52"/>
+      <x:c r="D2" s="124"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="53" t="str">
+      <x:c r="A3" s="125" t="str">
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
@@ -4324,12 +6322,12 @@
       <x:c r="C3" s="10" t="str">
         <x:v>Cursor Models &amp; Pricing docs</x:v>
       </x:c>
-      <x:c r="D3" s="54" t="str">
+      <x:c r="D3" s="126" t="str">
         <x:v>Explore all frontier coding models, usage pools, plan pricing, and per-model API rates.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="53" t="str">
+      <x:c r="A4" s="125" t="str">
         <x:v>Data extraction</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
@@ -4338,12 +6336,12 @@
       <x:c r="C4" s="10" t="str">
         <x:v>Parsed locally from the docs page bundle fetched during this session.</x:v>
       </x:c>
-      <x:c r="D4" s="54" t="str">
+      <x:c r="D4" s="126" t="str">
         <x:v>The workbook preserves visible and hidden metadata rows separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="53" t="str">
+      <x:c r="A5" s="125" t="str">
         <x:v>Sorting</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
@@ -4352,12 +6350,12 @@
       <x:c r="C5" s="10" t="str">
         <x:v>Calculated from editable assumptions.</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="126" t="str">
         <x:v>Change Assumptions!B5:B11 to adapt the estimate.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="53" t="str">
+      <x:c r="A6" s="125" t="str">
         <x:v>Simple Total $/1M</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
@@ -4366,12 +6364,12 @@
       <x:c r="C6" s="10" t="str">
         <x:v>A raw sum of published rate columns.</x:v>
       </x:c>
-      <x:c r="D6" s="54" t="str">
+      <x:c r="D6" s="126" t="str">
         <x:v>This is not a real bill by itself because workloads mix token types unevenly.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="53" t="str">
+      <x:c r="A7" s="125" t="str">
         <x:v>Estimated Blended $/1M</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
@@ -4380,12 +6378,12 @@
       <x:c r="C7" s="10" t="str">
         <x:v>Uses shares for uncached input, cache write, cache read, and output.</x:v>
       </x:c>
-      <x:c r="D7" s="54" t="str">
+      <x:c r="D7" s="126" t="str">
         <x:v>Designed as a practical cost-comparison sort key.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="53" t="str">
+      <x:c r="A8" s="125" t="str">
         <x:v>Teams note</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
@@ -4394,12 +6392,12 @@
       <x:c r="C8" s="10" t="str">
         <x:v>Set Assumptions!B11 to 1 to include the Teams non-Auto surcharge.</x:v>
       </x:c>
-      <x:c r="D8" s="54" t="str">
+      <x:c r="D8" s="126" t="str">
         <x:v>Default is off.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A9" s="53" t="str">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="125" t="str">
         <x:v>Max Mode note</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
@@ -4408,22 +6406,190 @@
       <x:c r="C9" s="10" t="str">
         <x:v>Rows are included where Cursor publishes different long-context rates.</x:v>
       </x:c>
-      <x:c r="D9" s="54" t="str">
+      <x:c r="D9" s="126" t="str">
         <x:v>Actual Max Mode availability and pricing may vary by plan.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="55" t="str">
+      <x:c r="A10" s="125" t="str">
         <x:v>Caveat</x:v>
       </x:c>
-      <x:c r="B10" s="56" t="str">
+      <x:c r="B10" s="10" t="str">
         <x:v>Rates change frequently</x:v>
       </x:c>
-      <x:c r="C10" s="56" t="str">
+      <x:c r="C10" s="10" t="str">
         <x:v>Refresh from Cursor docs before making a billing commitment.</x:v>
       </x:c>
-      <x:c r="D10" s="57" t="str">
+      <x:c r="D10" s="126" t="str">
         <x:v>This workbook is current as of the date shown in Assumptions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="125" t="str">
+        <x:v>Benchmark usage</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>Benchmark Guide / Benchmark Signals / Task Fit Matrix</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>Use benchmark evidence as a task-fit and escalation signal, not a ranking override.</x:v>
+      </x:c>
+      <x:c r="D11" s="126" t="str">
+        <x:v>Always combine benchmark evidence with Model Rates, task risk, verification strength, and project guidance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="125" t="str">
+        <x:v>CursorBench / Composer 2</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>https://arxiv.org/abs/2603.24477</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>CursorBench, Terminal-Bench, and SWE-bench Multilingual Composer 2 reported scores.</x:v>
+      </x:c>
+      <x:c r="D12" s="126" t="str">
+        <x:v>Used as Cursor-native agentic coding evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="125" t="str">
+        <x:v>Aider Polyglot</x:v>
+      </x:c>
+      <x:c r="B13" s="10" t="str">
+        <x:v>https://aider.chat/docs/leaderboards/</x:v>
+      </x:c>
+      <x:c r="C13" s="10" t="str">
+        <x:v>Leaderboard with score, cost, prompt tokens, and completion tokens.</x:v>
+      </x:c>
+      <x:c r="D13" s="126" t="str">
+        <x:v>Used for reasoning-level cost/reliability tradeoffs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="125" t="str">
+        <x:v>SWE-bench</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>https://www.swebench.com/</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>Official SWE-bench family overview and leaderboard.</x:v>
+      </x:c>
+      <x:c r="D14" s="126" t="str">
+        <x:v>Used for existing-repo issue-resolution task fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="125" t="str">
+        <x:v>SWE-bench Pro</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>https://arxiv.org/abs/2509.16941</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Long-horizon enterprise software engineering benchmark.</x:v>
+      </x:c>
+      <x:c r="D15" s="126" t="str">
+        <x:v>Used for broad architecture and multi-system escalation signals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="125" t="str">
+        <x:v>Terminal-Bench 2.0</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>https://www.tbench.ai/leaderboard/terminal-bench/2.0</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>Terminal-agent benchmark leaderboard.</x:v>
+      </x:c>
+      <x:c r="D16" s="126" t="str">
+        <x:v>Used for CLI, build, CI, deployment, and terminal-heavy work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="125" t="str">
+        <x:v>BigCodeBench</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>https://arxiv.org/abs/2406.15877</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>Broad code-generation benchmark requiring function calls and library/API use.</x:v>
+      </x:c>
+      <x:c r="D17" s="126" t="str">
+        <x:v>Used for API/library/tool-use task fit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="125" t="str">
+        <x:v>SWE-Lancer</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>https://openai.com/index/swe-lancer/</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="str">
+        <x:v>OpenAI benchmark built from freelance software engineering tasks.</x:v>
+      </x:c>
+      <x:c r="D18" s="126" t="str">
+        <x:v>Used for managerial and economically meaningful software task signals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="125" t="str">
+        <x:v>SWE-Bench Mobile</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>https://arxiv.org/abs/2602.09540</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="str">
+        <x:v>Production iOS/mobile software engineering benchmark.</x:v>
+      </x:c>
+      <x:c r="D19" s="126" t="str">
+        <x:v>Used for Apple-platform and mobile UI caution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="125" t="str">
+        <x:v>SpecBench</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>https://arxiv.org/abs/2605.30314</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="str">
+        <x:v>Specification-level software engineering benchmark.</x:v>
+      </x:c>
+      <x:c r="D20" s="126" t="str">
+        <x:v>Used for requirements, architecture, and design-review escalation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="125" t="str">
+        <x:v>SWE-Skills-Bench</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>https://arxiv.org/abs/2603.15401</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>Skill-injection benefit and token-overhead benchmark.</x:v>
+      </x:c>
+      <x:c r="D21" s="126" t="str">
+        <x:v>Used for plugin/skill minimalism.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="127" t="str">
+        <x:v>CORE-Bench</x:v>
+      </x:c>
+      <x:c r="B22" s="128" t="str">
+        <x:v>https://arxiv.org/abs/2606.11864</x:v>
+      </x:c>
+      <x:c r="C22" s="128" t="str">
+        <x:v>Repository code retrieval/localization benchmark.</x:v>
+      </x:c>
+      <x:c r="D22" s="129" t="str">
+        <x:v>Used for large-repo context and MAX Mode decisions.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>